<commit_message>
Fix РАГ -> RAG naming throughout scope docs
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/analysis/case-27-proekt-d8-skoup-i-voprosy.xlsx
+++ b/docs/analysis/case-27-proekt-d8-skoup-i-voprosy.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Волны проекта" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр платформы" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Скоуп — известное" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Структура РАГ-КХД-API-Users" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Структура RAG-КХД-API-Users" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Программа проекта" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Пример этапа" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Наши предложения" sheetId="8" state="visible" r:id="rId8"/>
@@ -668,7 +668,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Волна 1 «РАГ-документы» — что именно имеется в виду: (а) новые типы документов сверх пилотных двух коллекций, (б) улучшение качества/покрытия уже загруженного, или (в) отдельная новая коллекция под конкретную задачу/подразделение?</t>
+          <t>Волна 1 «RAG-документы» — что именно имеется в виду: (а) новые типы документов сверх пилотных двух коллекций, (б) улучшение качества/покрытия уже загруженного, или (в) отдельная новая коллекция под конкретную задачу/подразделение?</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>РАГ-документы</t>
+          <t>RAG-документы</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -2120,7 +2120,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Структура волн 1–2: РАГ, КХД, API на шине, пользователи</t>
+          <t>Структура волн 1–2: RAG, КХД, API на шине, пользователи</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2134,7 @@
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
-          <t>1. Структура РАГ (документные коллекции) — волна 1</t>
+          <t>1. Структура RAG (документные коллекции) — волна 1</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Волна 1 — РАГ-документы</t>
+          <t>Волна 1 — RAG-документы</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Rework D8 deck: architecture slide, per-wave checklist, refined questions
- Презентация: добавлен слайд архитектуры пилота (2/6), вопросы по
  волнам переведены из плоской таблицы в 3 карточки (Волна 1/2/3+),
  каждая по единому набору параметров — состав данных, витрины/
  коллекции, пользователи, роли; вопросы 6/7/12 из старой таблицы
  поглощены этим форматом. Обложка: убраны путь к xlsx и дата среза.
- Вопросы 8-11 (права доступа, кастомизация источников, персональные
  RAG-коллекции, упрощение регистрации) переформулированы по прямым
  уточнениям заказчика — синхронизировано в md/docx/xlsx/pptx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/analysis/case-27-proekt-d8-skoup-i-voprosy.xlsx
+++ b/docs/analysis/case-27-proekt-d8-skoup-i-voprosy.xlsx
@@ -990,7 +990,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Права доступа сотрудников сейчас фиксированы по статичному списку политик. Для проекта это должно стать динамическим (через таблицы/API из системы-источника прав)? Если да — какая система является источником истины по правам (HR-система, Bitrix24, отдельный IAM)?</t>
+          <t>Права доступа сотрудников сейчас фиксированы по статичному списку политик. Для проекта это должно стать динамическим через API — но нужна точная схема: права хранятся и администрируются внутри платформы, или платформа получает их из внешней системы через API и только применяет? Если второе — какая система источник истины и как часто права обновляются?</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Кастомизация выбора источников — нужна ли возможность подключать/отключать источники данных внутри компании прямо в режиме чата и через API, или фиксированный набор источников на пользователя/роль достаточен?</t>
+          <t>Кастомизация выбора источников — нужно уточнить, что имеется в виду: (а) подключение/отключение целых каталогов данных внутри домена компании, или (б) выбор персоны/профиля пользователя с отдельным набором прав доступа? Это разные по объёму реализации задачи.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr"/>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Персональные RAG-коллекции пользователей — нужна ли пользователям возможность самим создавать RAG-коллекции и делиться ими с коллегами?</t>
+          <t>Персональные RAG-коллекции пользователей — нужно уточнить механику: фильтр по документам внутри уже существующей коллекции, или отдельная новая коллекция, которую пользователь создаёт и наполняет сам?</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr"/>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Упрощение заведения пользователей — что именно сейчас неудобно в процессе добавления новых пользователей на стороне Д8? Нужен конкретный сценарий.</t>
+          <t>Упрощение заведения пользователей — нужен не общий запрос, а конкретный кейс: как должен выглядеть процесс пошагово (кто инициирует, какие поля, кто подтверждает).</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Turn wave goal/criteria into questions to the customer, add proposals slide
- Волновые карточки (пптx) и вопросы 2/4/8 (md) больше не содержат
  наших формулировок цели/критерия — это прямые вопросы к Д8: какая
  цель волны и какой критерий её достижения. Добавлено в xlsx (новые
  вопросы №2, №5, №9) и синхронизировано в md/docx (вопросы 1-18,
  полная renumbering всех перекрёстных ссылок).
- Новый слайд «Наши предложения» (6/7) — 6 рабочих позиций по
  умолчанию из §6 документа, на основе программы проекта.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DpSN8JwCJ3tg3JVUadr2zE
</commit_message>
<xml_diff>
--- a/docs/analysis/case-27-proekt-d8-skoup-i-voprosy.xlsx
+++ b/docs/analysis/case-27-proekt-d8-skoup-i-voprosy.xlsx
@@ -572,7 +572,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Зависит от ответов на вопросы №1 (волна 1), №4–6 (ESB/КХД)</t>
+          <t>Зависит от ответов на вопросы №1 (волна 1), №6–8 (ESB/КХД)</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Зависит от вопроса №2 (детальный состав работ) и вопросов №4–6 (список витрин/API), №8 (динамические права — как gate для чувствительных волн)</t>
+          <t>Зависит от вопроса №3 (детальный состав работ) и вопросов №6–8 (список витрин/API), №11 (динамические права — как gate для чувствительных волн)</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Зависит от вопроса №12 (кто владелец процесса со стороны Д8)</t>
+          <t>Зависит от вопроса №15 (кто владелец процесса со стороны Д8)</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -824,12 +824,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Волна 2 — нужен детальный состав работ: список конкретных витрин/API, которые нужно добавить в ESB и КХД (не только общее направление «расширить»).</t>
+          <t>Цель и критерий волны 1 — какой результат для бизнеса должна дать волна 1? По каким признакам вы будете считать её завершённой и успешной?</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Собрать вместе с заказчиком на отдельной встрече — состав работ определяет и срок, и трудоёмкость волны 2.</t>
+          <t>Это должен сформулировать сам Д8 — не готовая формулировка от нас, а прямой запрос к заказчику.</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr"/>
@@ -848,17 +848,21 @@
           <t>Волны проекта</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Высокий</t>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Критичный</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Волна 3 и далее — есть ли уже примерное направление (роли, новые источники, промышленная эксплуатация), или это открытый вопрос до завершения волны 2?</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr"/>
+          <t>Волна 2 — нужен детальный состав работ: список конкретных витрин/API, которые нужно добавить в ESB и КХД (не только общее направление «расширить»).</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Собрать вместе с заказчиком на отдельной встрече — состав работ определяет и срок, и трудоёмкость волны 2.</t>
+        </is>
+      </c>
       <c r="F6" s="8" t="inlineStr"/>
       <c r="G6" s="8" t="inlineStr">
         <is>
@@ -872,7 +876,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Интеграция (ESB/КХД, волна 2)</t>
+          <t>Волны проекта</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -882,7 +886,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Какие конкретно витрины данных нужно добавить в ESB сверх текущего среза CRM (Bitrix24)? Список витрин с владельцами на стороне Д8.</t>
+          <t>Волна 3 и далее — есть ли уже примерное направление (роли, новые источники, промышленная эксплуатация), или это открытый вопрос до завершения волны 2?</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
@@ -899,7 +903,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Интеграция (ESB/КХД, волна 2)</t>
+          <t>Волны проекта</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -909,7 +913,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Какие конкретно API нужно открыть через шину — по каждому: система-источник, формат (REST/SOAP/др.), кто на стороне Д8 отвечает за контракт API.</t>
+          <t>Цель и критерий волны 3+ — когда направление определится, какая бизнес-цель будет стоять за ней, и какими критериями вы будете руководствоваться при выборе?</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr"/>
@@ -936,7 +940,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>КХД — расширяется ли состав таблиц/витрин внутри самого хранилища, или его периметр остаётся как в пилоте?</t>
+          <t>Какие конкретно витрины данных нужно добавить в ESB сверх текущего среза CRM (Bitrix24)? Список витрин с владельцами на стороне Д8.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
@@ -953,17 +957,17 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Права доступа и роли</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Нормальный</t>
+          <t>Интеграция (ESB/КХД, волна 2)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Реальная оргструктура для проекта: список подразделений/ролей с числом пользователей в каждой (не гипотетическая таблица из мастер-ТЗ, а факт) — нужна для карты волн 3+.</t>
+          <t>Какие конкретно API нужно открыть через шину — по каждому: система-источник, формат (REST/SOAP/др.), кто на стороне Д8 отвечает за контракт API.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr"/>
@@ -980,7 +984,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Права доступа и роли</t>
+          <t>Интеграция (ESB/КХД, волна 2)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -990,14 +994,10 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Права доступа сотрудников сейчас фиксированы по статичному списку политик. Для проекта это должно стать динамическим через API — но нужна точная схема: права хранятся и администрируются внутри платформы, или платформа получает их из внешней системы через API и только применяет? Если второе — какая система источник истины и как часто права обновляются?</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Не блокировать волну 2 (запускать на статичной модели, как в пилоте), но зафиксировать как gate для волн с чувствительными данными (комплаенс, бэк-офис). Платформа тоже отметила это «Уточнить у заказчика» — ждёт ответа с обеих сторон.</t>
-        </is>
-      </c>
+          <t>КХД — расширяется ли состав таблиц/витрин внутри самого хранилища, или его периметр остаётся как в пилоте?</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="8" t="inlineStr"/>
       <c r="G11" s="8" t="inlineStr">
         <is>
@@ -1011,17 +1011,17 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Платформенные возможности</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Нормальный</t>
+          <t>Интеграция (ESB/КХД, волна 2)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Кастомизация выбора источников — нужно уточнить, что имеется в виду: (а) подключение/отключение целых каталогов данных внутри домена компании, или (б) выбор персоны/профиля пользователя с отдельным набором прав доступа? Это разные по объёму реализации задачи.</t>
+          <t>Цель и критерий волны 2 — какую бизнес-задачу решает расширение ESB/КХД? По какому набору проверок/сценариев вы примете волну 2 как завершённую?</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr"/>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Платформенные возможности</t>
+          <t>Права доступа и роли</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Персональные RAG-коллекции пользователей — нужно уточнить механику: фильтр по документам внутри уже существующей коллекции, или отдельная новая коллекция, которую пользователь создаёт и наполняет сам?</t>
+          <t>Реальная оргструктура для проекта: список подразделений/ролей с числом пользователей в каждой (не гипотетическая таблица из мастер-ТЗ, а факт) — нужна для карты волн 3+.</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr"/>
@@ -1065,20 +1065,24 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Платформенные возможности</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Нормальный</t>
+          <t>Права доступа и роли</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Упрощение заведения пользователей — нужен не общий запрос, а конкретный кейс: как должен выглядеть процесс пошагово (кто инициирует, какие поля, кто подтверждает).</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr"/>
+          <t>Права доступа сотрудников сейчас фиксированы по статичному списку политик. Для проекта это должно стать динамическим через API — но нужна точная схема: права хранятся и администрируются внутри платформы, или платформа получает их из внешней системы через API и только применяет? Если второе — какая система источник истины и как часто права обновляются?</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Не блокировать волну 2 (запускать на статичной модели, как в пилоте), но зафиксировать как gate для волн с чувствительными данными (комплаенс, бэк-офис). Платформа тоже отметила это «Уточнить у заказчика» — ждёт ответа с обеих сторон.</t>
+        </is>
+      </c>
       <c r="F14" s="8" t="inlineStr"/>
       <c r="G14" s="8" t="inlineStr">
         <is>
@@ -1092,7 +1096,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Общее по проекту</t>
+          <t>Платформенные возможности</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1102,12 +1106,93 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Кто со стороны Д8 — новый владелец процесса на фазе П4 (промышленная эксплуатация)? Тот же технический контакт, что в пилоте, или отдельная выделенная роль/команда?</t>
+          <t>Кастомизация выбора источников — нужно уточнить, что имеется в виду: (а) подключение/отключение целых каталогов данных внутри домена компании, или (б) выбор персоны/профиля пользователя с отдельным набором прав доступа? Это разные по объёму реализации задачи.</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="8" t="inlineStr"/>
       <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Требует проработки</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Платформенные возможности</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Нормальный</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Персональные RAG-коллекции пользователей — нужно уточнить механику: фильтр по документам внутри уже существующей коллекции, или отдельная новая коллекция, которую пользователь создаёт и наполняет сам?</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Требует проработки</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Платформенные возможности</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Нормальный</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Упрощение заведения пользователей — нужен не общий запрос, а конкретный кейс: как должен выглядеть процесс пошагово (кто инициирует, какие поля, кто подтверждает).</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Требует проработки</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Общее по проекту</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Нормальный</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Кто со стороны Д8 — новый владелец процесса на фазе П4 (промышленная эксплуатация)? Тот же технический контакт, что в пилоте, или отдельная выделенная роль/команда?</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr">
         <is>
           <t>Требует проработки</t>
         </is>

</xml_diff>